<commit_message>
Add StockSeeder,ClassementSeeder,StockImport. Modifying Table classement(Model,Contr,Migration)
</commit_message>
<xml_diff>
--- a/backend-erp/database/seeders/data/Stocks.xlsx
+++ b/backend-erp/database/seeders/data/Stocks.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Compagnie Malagasy de Plastique\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3A979EC-C319-4F45-B45C-08D9F21447C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{19D14CF1-44C9-4EA2-AE0C-020E7E59462F}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -50,9 +44,6 @@
     <t>classement_id</t>
   </si>
   <si>
-    <t>stocks-total</t>
-  </si>
-  <si>
     <t>produit</t>
   </si>
   <si>
@@ -297,13 +288,16 @@
   </si>
   <si>
     <t>1L Carré Strié</t>
+  </si>
+  <si>
+    <t>stocks_total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -412,7 +406,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -464,7 +458,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -678,26 +672,26 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF9D992C-31F4-4751-A55B-DAB24050CD46}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F85"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.75" customWidth="1"/>
+    <col min="2" max="2" width="11.125" customWidth="1"/>
     <col min="3" max="3" width="31" style="2" customWidth="1"/>
     <col min="4" max="4" width="26" style="3" customWidth="1"/>
-    <col min="5" max="5" width="6.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" customWidth="1"/>
+    <col min="5" max="5" width="6.625" customWidth="1"/>
+    <col min="6" max="6" width="11.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -708,27 +702,27 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="1">
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2">
         <v>973</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -737,18 +731,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" s="2">
         <v>974</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -757,18 +751,18 @@
         <v>7746</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" s="2">
         <v>975</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -777,18 +771,18 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" s="1">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" s="2">
         <v>976</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -797,18 +791,18 @@
         <v>4329</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" s="1">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" s="2">
         <v>977</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -817,18 +811,18 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6">
       <c r="A7" s="1">
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" s="2">
         <v>978</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -837,18 +831,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6">
       <c r="A8" s="1">
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="2">
         <v>979</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -857,18 +851,18 @@
         <v>2730</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6">
       <c r="A9" s="1">
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" s="2">
         <v>980</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -877,18 +871,18 @@
         <v>581</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6">
       <c r="A10" s="1">
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" s="2">
         <v>981</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -897,18 +891,18 @@
         <v>4428</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6">
       <c r="A11" s="1">
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C11" s="2">
         <v>982</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -917,18 +911,18 @@
         <v>826</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6">
       <c r="A12" s="1">
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C12" s="2">
         <v>983</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -937,18 +931,18 @@
         <v>7298</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6">
       <c r="A13" s="1">
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13" s="2">
         <v>984</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -957,18 +951,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6">
       <c r="A14" s="1">
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2">
         <v>985</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -977,18 +971,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6">
       <c r="A15" s="1">
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2">
         <v>986</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -997,18 +991,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6">
       <c r="A16" s="1">
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C16" s="2">
         <v>987</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -1017,18 +1011,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6">
       <c r="A17" s="1">
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C17" s="2">
         <v>988</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -1037,18 +1031,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6">
       <c r="A18" s="1">
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C18" s="2">
         <v>989</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -1057,18 +1051,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6">
       <c r="A19" s="1">
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C19" s="2">
         <v>990</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -1077,18 +1071,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6">
       <c r="A20" s="1">
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20" s="2">
         <v>991</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1097,18 +1091,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6">
       <c r="A21" s="1">
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C21" s="2">
         <v>992</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -1117,18 +1111,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6">
       <c r="A22" s="1">
         <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C22" s="2">
         <v>993</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -1137,18 +1131,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6">
       <c r="A23" s="1">
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C23" s="2">
         <v>994</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -1157,18 +1151,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6">
       <c r="A24" s="1">
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C24" s="2">
         <v>995</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -1177,18 +1171,18 @@
         <v>2765</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6">
       <c r="A25" s="1">
         <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C25" s="2">
         <v>996</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -1197,18 +1191,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6">
       <c r="A26" s="1">
         <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" s="2">
         <v>997</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -1217,18 +1211,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6">
       <c r="A27" s="1">
         <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" s="2">
         <v>998</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -1237,18 +1231,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6">
       <c r="A28" s="1">
         <v>2</v>
       </c>
       <c r="B28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28" s="2">
         <v>999</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -1257,18 +1251,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6">
       <c r="A29" s="1">
         <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" s="2">
         <v>1000</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -1277,18 +1271,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6">
       <c r="A30" s="1">
         <v>2</v>
       </c>
       <c r="B30" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C30" s="2">
         <v>1001</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -1297,18 +1291,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6">
       <c r="A31" s="1">
         <v>2</v>
       </c>
       <c r="B31" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C31" s="2">
         <v>1002</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -1317,18 +1311,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6">
       <c r="A32" s="1">
         <v>2</v>
       </c>
       <c r="B32" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C32" s="2">
         <v>1003</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -1337,18 +1331,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6">
       <c r="A33" s="1">
         <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C33" s="2">
         <v>1004</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -1357,18 +1351,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6">
       <c r="A34" s="1">
         <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C34" s="2">
         <v>1005</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -1377,18 +1371,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6">
       <c r="A35" s="1">
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C35" s="2">
         <v>1006</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -1397,18 +1391,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6">
       <c r="A36" s="1">
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C36" s="2">
         <v>1007</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -1417,18 +1411,18 @@
         <v>1327</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6">
       <c r="A37" s="1">
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C37" s="2">
         <v>1008</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -1437,18 +1431,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6">
       <c r="A38" s="1">
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C38" s="2">
         <v>1009</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -1457,18 +1451,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6">
       <c r="A39" s="1">
         <v>2</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C39" s="2">
         <v>1010</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -1477,18 +1471,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6">
       <c r="A40" s="1">
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C40" s="2">
         <v>1011</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -1497,18 +1491,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6">
       <c r="A41" s="1">
         <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C41" s="2">
         <v>1012</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -1517,18 +1511,18 @@
         <v>742</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6">
       <c r="A42" s="1">
         <v>2</v>
       </c>
       <c r="B42" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C42" s="2">
         <v>1013</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -1537,18 +1531,18 @@
         <v>2247</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6">
       <c r="A43" s="1">
         <v>2</v>
       </c>
       <c r="B43" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C43" s="2">
         <v>1014</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -1557,18 +1551,18 @@
         <v>712</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6">
       <c r="A44" s="1">
         <v>2</v>
       </c>
       <c r="B44" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C44" s="2">
         <v>1015</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -1577,18 +1571,18 @@
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6">
       <c r="A45" s="1">
         <v>2</v>
       </c>
       <c r="B45" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C45" s="2">
         <v>1016</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -1597,18 +1591,18 @@
         <v>78</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6">
       <c r="A46" s="1">
         <v>2</v>
       </c>
       <c r="B46" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C46" s="2">
         <v>1017</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -1617,18 +1611,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6">
       <c r="A47" s="1">
         <v>2</v>
       </c>
       <c r="B47" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C47" s="2">
         <v>1018</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -1637,18 +1631,18 @@
         <v>1998</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6">
       <c r="A48" s="1">
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C48" s="2">
         <v>1019</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -1657,18 +1651,18 @@
         <v>16266</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6">
       <c r="A49" s="1">
         <v>2</v>
       </c>
       <c r="B49" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C49" s="2">
         <v>1020</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -1677,18 +1671,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6">
       <c r="A50" s="1">
         <v>2</v>
       </c>
       <c r="B50" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C50" s="2">
         <v>1021</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -1697,18 +1691,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6">
       <c r="A51" s="1">
         <v>2</v>
       </c>
       <c r="B51" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C51" s="2">
         <v>1022</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -1717,18 +1711,18 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6">
       <c r="A52" s="1">
         <v>2</v>
       </c>
       <c r="B52" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C52" s="2">
         <v>1023</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -1737,18 +1731,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6">
       <c r="A53" s="1">
         <v>2</v>
       </c>
       <c r="B53" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C53" s="2">
         <v>1024</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -1757,18 +1751,18 @@
         <v>385</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6">
       <c r="A54" s="1">
         <v>2</v>
       </c>
       <c r="B54" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C54" s="2">
         <v>1025</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -1777,18 +1771,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6">
       <c r="A55" s="1">
         <v>2</v>
       </c>
       <c r="B55" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C55" s="2">
         <v>1026</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -1797,18 +1791,18 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6">
       <c r="A56" s="1">
         <v>2</v>
       </c>
       <c r="B56" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C56" s="2">
         <v>1027</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -1817,18 +1811,18 @@
         <v>141</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6">
       <c r="A57" s="1">
         <v>2</v>
       </c>
       <c r="B57" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C57" s="2">
         <v>1028</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -1837,18 +1831,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6">
       <c r="A58" s="1">
         <v>2</v>
       </c>
       <c r="B58" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C58" s="2">
         <v>1029</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -1857,18 +1851,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6">
       <c r="A59" s="1">
         <v>2</v>
       </c>
       <c r="B59" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C59" s="2">
         <v>1030</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -1877,18 +1871,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6">
       <c r="A60" s="1">
         <v>2</v>
       </c>
       <c r="B60" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C60" s="2">
         <v>1031</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -1897,18 +1891,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6">
       <c r="A61" s="1">
         <v>2</v>
       </c>
       <c r="B61" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C61" s="2">
         <v>1032</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -1917,18 +1911,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6">
       <c r="A62" s="1">
         <v>2</v>
       </c>
       <c r="B62" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C62" s="2">
         <v>1033</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -1937,18 +1931,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6">
       <c r="A63" s="1">
         <v>2</v>
       </c>
       <c r="B63" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C63" s="2">
         <v>1034</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -1957,18 +1951,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6">
       <c r="A64" s="1">
         <v>2</v>
       </c>
       <c r="B64" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C64" s="2">
         <v>1035</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -1977,18 +1971,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6">
       <c r="A65" s="1">
         <v>2</v>
       </c>
       <c r="B65" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C65" s="2">
         <v>1036</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -1997,18 +1991,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6">
       <c r="A66" s="1">
         <v>2</v>
       </c>
       <c r="B66" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C66" s="2">
         <v>1037</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -2017,18 +2011,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6">
       <c r="A67" s="1">
         <v>2</v>
       </c>
       <c r="B67" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C67" s="2">
         <v>1038</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -2037,18 +2031,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6">
       <c r="A68" s="1">
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C68" s="2">
         <v>1039</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E68">
         <v>1</v>
@@ -2057,18 +2051,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6">
       <c r="A69" s="1">
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C69" s="2">
         <v>1040</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -2077,18 +2071,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6">
       <c r="A70" s="1">
         <v>2</v>
       </c>
       <c r="B70" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C70" s="2">
         <v>1041</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -2097,18 +2091,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6">
       <c r="A71" s="1">
         <v>2</v>
       </c>
       <c r="B71" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C71" s="2">
         <v>1042</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -2117,18 +2111,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6">
       <c r="A72" s="1">
         <v>2</v>
       </c>
       <c r="B72" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C72" s="2">
         <v>1043</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -2137,18 +2131,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6">
       <c r="A73" s="1">
         <v>2</v>
       </c>
       <c r="B73" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C73" s="2">
         <v>1044</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -2157,18 +2151,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6">
       <c r="A74" s="1">
         <v>2</v>
       </c>
       <c r="B74" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C74" s="2">
         <v>1045</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -2177,18 +2171,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6">
       <c r="A75" s="1">
         <v>2</v>
       </c>
       <c r="B75" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C75" s="2">
         <v>1046</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -2197,18 +2191,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6">
       <c r="A76" s="1">
         <v>2</v>
       </c>
       <c r="B76" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C76" s="2">
         <v>1047</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E76">
         <v>1</v>
@@ -2217,18 +2211,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6">
       <c r="A77" s="1">
         <v>2</v>
       </c>
       <c r="B77" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C77" s="2">
         <v>1048</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -2237,18 +2231,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6">
       <c r="A78" s="1">
         <v>2</v>
       </c>
       <c r="B78" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C78" s="2">
         <v>1049</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -2257,18 +2251,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6">
       <c r="A79" s="1">
         <v>2</v>
       </c>
       <c r="B79" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C79" s="2">
         <v>1050</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -2277,18 +2271,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6">
       <c r="A80" s="1">
         <v>2</v>
       </c>
       <c r="B80" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C80" s="2">
         <v>1051</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -2297,18 +2291,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6">
       <c r="A81" s="1">
         <v>2</v>
       </c>
       <c r="B81" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C81" s="2">
         <v>1052</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -2317,18 +2311,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6">
       <c r="A82" s="1">
         <v>2</v>
       </c>
       <c r="B82" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C82" s="2">
         <v>1053</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -2337,13 +2331,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6">
       <c r="A83" s="1"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6">
       <c r="A84" s="1"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6">
       <c r="A85" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding Module Stock and Production
</commit_message>
<xml_diff>
--- a/backend-erp/database/seeders/data/Stocks.xlsx
+++ b/backend-erp/database/seeders/data/Stocks.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="92">
   <si>
     <t>location_id</t>
   </si>
@@ -291,6 +291,21 @@
   </si>
   <si>
     <t>stocks_total</t>
+  </si>
+  <si>
+    <t>Huilerie 1L</t>
+  </si>
+  <si>
+    <t>Bassine coulleur assorti</t>
+  </si>
+  <si>
+    <t>Huilerie 250 ML</t>
+  </si>
+  <si>
+    <t>Huilerie 500 ML</t>
+  </si>
+  <si>
+    <t>Seau Vert C</t>
   </si>
 </sst>
 </file>
@@ -680,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.75" customWidth="1"/>
@@ -719,7 +734,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="2">
-        <v>973</v>
+        <v>1</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>6</v>
@@ -739,7 +754,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="2">
-        <v>974</v>
+        <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>7</v>
@@ -759,7 +774,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="2">
-        <v>975</v>
+        <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>8</v>
@@ -779,7 +794,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="2">
-        <v>976</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
@@ -799,7 +814,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="2">
-        <v>977</v>
+        <v>5</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>10</v>
@@ -819,7 +834,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="2">
-        <v>978</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>11</v>
@@ -839,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="2">
-        <v>979</v>
+        <v>7</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>12</v>
@@ -859,7 +874,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="2">
-        <v>980</v>
+        <v>8</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>13</v>
@@ -879,7 +894,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="2">
-        <v>981</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>14</v>
@@ -899,7 +914,7 @@
         <v>4</v>
       </c>
       <c r="C11" s="2">
-        <v>982</v>
+        <v>10</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>15</v>
@@ -919,7 +934,7 @@
         <v>4</v>
       </c>
       <c r="C12" s="2">
-        <v>983</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>16</v>
@@ -939,7 +954,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="2">
-        <v>984</v>
+        <v>12</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>17</v>
@@ -959,7 +974,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="2">
-        <v>985</v>
+        <v>13</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>18</v>
@@ -979,7 +994,7 @@
         <v>4</v>
       </c>
       <c r="C15" s="2">
-        <v>986</v>
+        <v>14</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>19</v>
@@ -999,7 +1014,7 @@
         <v>4</v>
       </c>
       <c r="C16" s="2">
-        <v>987</v>
+        <v>15</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>20</v>
@@ -1019,7 +1034,7 @@
         <v>4</v>
       </c>
       <c r="C17" s="2">
-        <v>988</v>
+        <v>16</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>21</v>
@@ -1039,7 +1054,7 @@
         <v>4</v>
       </c>
       <c r="C18" s="2">
-        <v>989</v>
+        <v>17</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>22</v>
@@ -1059,7 +1074,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="2">
-        <v>990</v>
+        <v>18</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>23</v>
@@ -1079,7 +1094,7 @@
         <v>4</v>
       </c>
       <c r="C20" s="2">
-        <v>991</v>
+        <v>19</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>24</v>
@@ -1099,7 +1114,7 @@
         <v>4</v>
       </c>
       <c r="C21" s="2">
-        <v>992</v>
+        <v>20</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>25</v>
@@ -1119,7 +1134,7 @@
         <v>4</v>
       </c>
       <c r="C22" s="2">
-        <v>993</v>
+        <v>21</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>26</v>
@@ -1139,7 +1154,7 @@
         <v>4</v>
       </c>
       <c r="C23" s="2">
-        <v>994</v>
+        <v>22</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>27</v>
@@ -1159,7 +1174,7 @@
         <v>4</v>
       </c>
       <c r="C24" s="2">
-        <v>995</v>
+        <v>23</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>28</v>
@@ -1179,7 +1194,7 @@
         <v>4</v>
       </c>
       <c r="C25" s="2">
-        <v>996</v>
+        <v>24</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>29</v>
@@ -1199,7 +1214,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="2">
-        <v>997</v>
+        <v>25</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>30</v>
@@ -1219,7 +1234,7 @@
         <v>4</v>
       </c>
       <c r="C27" s="2">
-        <v>998</v>
+        <v>26</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>31</v>
@@ -1239,7 +1254,7 @@
         <v>4</v>
       </c>
       <c r="C28" s="2">
-        <v>999</v>
+        <v>27</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>32</v>
@@ -1259,7 +1274,7 @@
         <v>4</v>
       </c>
       <c r="C29" s="2">
-        <v>1000</v>
+        <v>28</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>33</v>
@@ -1279,7 +1294,7 @@
         <v>4</v>
       </c>
       <c r="C30" s="2">
-        <v>1001</v>
+        <v>29</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>34</v>
@@ -1299,7 +1314,7 @@
         <v>4</v>
       </c>
       <c r="C31" s="2">
-        <v>1002</v>
+        <v>30</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>35</v>
@@ -1319,7 +1334,7 @@
         <v>4</v>
       </c>
       <c r="C32" s="2">
-        <v>1003</v>
+        <v>31</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>36</v>
@@ -1339,7 +1354,7 @@
         <v>4</v>
       </c>
       <c r="C33" s="2">
-        <v>1004</v>
+        <v>32</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>37</v>
@@ -1359,7 +1374,7 @@
         <v>4</v>
       </c>
       <c r="C34" s="2">
-        <v>1005</v>
+        <v>33</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>38</v>
@@ -1379,7 +1394,7 @@
         <v>4</v>
       </c>
       <c r="C35" s="2">
-        <v>1006</v>
+        <v>34</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>39</v>
@@ -1399,7 +1414,7 @@
         <v>4</v>
       </c>
       <c r="C36" s="2">
-        <v>1007</v>
+        <v>35</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>40</v>
@@ -1419,7 +1434,7 @@
         <v>4</v>
       </c>
       <c r="C37" s="2">
-        <v>1008</v>
+        <v>36</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>41</v>
@@ -1439,7 +1454,7 @@
         <v>4</v>
       </c>
       <c r="C38" s="2">
-        <v>1009</v>
+        <v>37</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>42</v>
@@ -1459,7 +1474,7 @@
         <v>4</v>
       </c>
       <c r="C39" s="2">
-        <v>1010</v>
+        <v>38</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>43</v>
@@ -1479,7 +1494,7 @@
         <v>4</v>
       </c>
       <c r="C40" s="2">
-        <v>1011</v>
+        <v>39</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>44</v>
@@ -1499,7 +1514,7 @@
         <v>4</v>
       </c>
       <c r="C41" s="2">
-        <v>1012</v>
+        <v>40</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>45</v>
@@ -1519,7 +1534,7 @@
         <v>4</v>
       </c>
       <c r="C42" s="2">
-        <v>1013</v>
+        <v>41</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>46</v>
@@ -1539,7 +1554,7 @@
         <v>4</v>
       </c>
       <c r="C43" s="2">
-        <v>1014</v>
+        <v>42</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>47</v>
@@ -1559,7 +1574,7 @@
         <v>4</v>
       </c>
       <c r="C44" s="2">
-        <v>1015</v>
+        <v>43</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>48</v>
@@ -1579,7 +1594,7 @@
         <v>4</v>
       </c>
       <c r="C45" s="2">
-        <v>1016</v>
+        <v>44</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>49</v>
@@ -1599,7 +1614,7 @@
         <v>4</v>
       </c>
       <c r="C46" s="2">
-        <v>1017</v>
+        <v>45</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>50</v>
@@ -1619,7 +1634,7 @@
         <v>4</v>
       </c>
       <c r="C47" s="2">
-        <v>1018</v>
+        <v>46</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>51</v>
@@ -1639,7 +1654,7 @@
         <v>4</v>
       </c>
       <c r="C48" s="2">
-        <v>1019</v>
+        <v>47</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>52</v>
@@ -1659,7 +1674,7 @@
         <v>4</v>
       </c>
       <c r="C49" s="2">
-        <v>1020</v>
+        <v>48</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>53</v>
@@ -1679,7 +1694,7 @@
         <v>4</v>
       </c>
       <c r="C50" s="2">
-        <v>1021</v>
+        <v>49</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>54</v>
@@ -1699,7 +1714,7 @@
         <v>4</v>
       </c>
       <c r="C51" s="2">
-        <v>1022</v>
+        <v>50</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>55</v>
@@ -1719,7 +1734,7 @@
         <v>4</v>
       </c>
       <c r="C52" s="2">
-        <v>1023</v>
+        <v>51</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>56</v>
@@ -1739,7 +1754,7 @@
         <v>4</v>
       </c>
       <c r="C53" s="2">
-        <v>1024</v>
+        <v>52</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>57</v>
@@ -1759,7 +1774,7 @@
         <v>4</v>
       </c>
       <c r="C54" s="2">
-        <v>1025</v>
+        <v>53</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>58</v>
@@ -1779,7 +1794,7 @@
         <v>4</v>
       </c>
       <c r="C55" s="2">
-        <v>1026</v>
+        <v>54</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>59</v>
@@ -1799,7 +1814,7 @@
         <v>4</v>
       </c>
       <c r="C56" s="2">
-        <v>1027</v>
+        <v>55</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>60</v>
@@ -1819,7 +1834,7 @@
         <v>4</v>
       </c>
       <c r="C57" s="2">
-        <v>1028</v>
+        <v>56</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>61</v>
@@ -1839,7 +1854,7 @@
         <v>4</v>
       </c>
       <c r="C58" s="2">
-        <v>1029</v>
+        <v>57</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>62</v>
@@ -1859,7 +1874,7 @@
         <v>4</v>
       </c>
       <c r="C59" s="2">
-        <v>1030</v>
+        <v>58</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>63</v>
@@ -1879,7 +1894,7 @@
         <v>4</v>
       </c>
       <c r="C60" s="2">
-        <v>1031</v>
+        <v>59</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>64</v>
@@ -1899,7 +1914,7 @@
         <v>4</v>
       </c>
       <c r="C61" s="2">
-        <v>1032</v>
+        <v>60</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>65</v>
@@ -1919,7 +1934,7 @@
         <v>4</v>
       </c>
       <c r="C62" s="2">
-        <v>1033</v>
+        <v>61</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>66</v>
@@ -1939,10 +1954,10 @@
         <v>4</v>
       </c>
       <c r="C63" s="2">
-        <v>1034</v>
+        <v>62</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -1959,7 +1974,7 @@
         <v>4</v>
       </c>
       <c r="C64" s="2">
-        <v>1035</v>
+        <v>63</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>67</v>
@@ -1979,7 +1994,7 @@
         <v>4</v>
       </c>
       <c r="C65" s="2">
-        <v>1036</v>
+        <v>64</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>68</v>
@@ -1999,7 +2014,7 @@
         <v>4</v>
       </c>
       <c r="C66" s="2">
-        <v>1037</v>
+        <v>65</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>69</v>
@@ -2019,7 +2034,7 @@
         <v>4</v>
       </c>
       <c r="C67" s="2">
-        <v>1038</v>
+        <v>66</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>70</v>
@@ -2039,7 +2054,7 @@
         <v>4</v>
       </c>
       <c r="C68" s="2">
-        <v>1039</v>
+        <v>67</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>71</v>
@@ -2059,7 +2074,7 @@
         <v>4</v>
       </c>
       <c r="C69" s="2">
-        <v>1040</v>
+        <v>68</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>72</v>
@@ -2079,7 +2094,7 @@
         <v>4</v>
       </c>
       <c r="C70" s="2">
-        <v>1041</v>
+        <v>69</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>73</v>
@@ -2099,7 +2114,7 @@
         <v>4</v>
       </c>
       <c r="C71" s="2">
-        <v>1042</v>
+        <v>70</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>74</v>
@@ -2119,7 +2134,7 @@
         <v>4</v>
       </c>
       <c r="C72" s="2">
-        <v>1043</v>
+        <v>71</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>75</v>
@@ -2139,7 +2154,7 @@
         <v>4</v>
       </c>
       <c r="C73" s="2">
-        <v>1044</v>
+        <v>72</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>76</v>
@@ -2159,7 +2174,7 @@
         <v>4</v>
       </c>
       <c r="C74" s="2">
-        <v>1045</v>
+        <v>73</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>77</v>
@@ -2179,7 +2194,7 @@
         <v>4</v>
       </c>
       <c r="C75" s="2">
-        <v>1046</v>
+        <v>74</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>78</v>
@@ -2199,7 +2214,7 @@
         <v>4</v>
       </c>
       <c r="C76" s="2">
-        <v>1047</v>
+        <v>75</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>79</v>
@@ -2219,7 +2234,7 @@
         <v>4</v>
       </c>
       <c r="C77" s="2">
-        <v>1048</v>
+        <v>76</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>80</v>
@@ -2239,7 +2254,7 @@
         <v>4</v>
       </c>
       <c r="C78" s="2">
-        <v>1049</v>
+        <v>77</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>81</v>
@@ -2259,7 +2274,7 @@
         <v>4</v>
       </c>
       <c r="C79" s="2">
-        <v>1050</v>
+        <v>78</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>82</v>
@@ -2279,7 +2294,7 @@
         <v>4</v>
       </c>
       <c r="C80" s="2">
-        <v>1051</v>
+        <v>79</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>83</v>
@@ -2299,7 +2314,7 @@
         <v>4</v>
       </c>
       <c r="C81" s="2">
-        <v>1052</v>
+        <v>80</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>84</v>
@@ -2319,7 +2334,7 @@
         <v>4</v>
       </c>
       <c r="C82" s="2">
-        <v>1053</v>
+        <v>81</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>85</v>
@@ -2332,13 +2347,84 @@
       </c>
     </row>
     <row r="83" spans="1:6">
-      <c r="A83" s="1"/>
+      <c r="A83" s="1">
+        <v>2</v>
+      </c>
+      <c r="B83" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" s="2">
+        <v>82</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
+      <c r="F83">
+        <v>34</v>
+      </c>
     </row>
     <row r="84" spans="1:6">
-      <c r="A84" s="1"/>
+      <c r="A84" s="1">
+        <v>2</v>
+      </c>
+      <c r="B84" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" s="2">
+        <v>83</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
     </row>
     <row r="85" spans="1:6">
-      <c r="A85" s="1"/>
+      <c r="A85" s="1">
+        <v>2</v>
+      </c>
+      <c r="B85" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="2">
+        <v>84</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85">
+        <v>5238</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" s="1">
+        <v>2</v>
+      </c>
+      <c r="B86" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" s="2">
+        <v>85</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86">
+        <v>392</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Module Factures, Delivery, Command
</commit_message>
<xml_diff>
--- a/backend-erp/database/seeders/data/Stocks.xlsx
+++ b/backend-erp/database/seeders/data/Stocks.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="brouilllon" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="144525"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="163">
   <si>
     <t>location_id</t>
   </si>
@@ -306,6 +307,219 @@
   </si>
   <si>
     <t>Seau Vert C</t>
+  </si>
+  <si>
+    <t>Bouchon HDPE Fanta Orange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 19 gr Clair Dmag </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 19gr Clair Husky </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 19 gr Blanc </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 36gr Husky </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 36 gr Toshiba </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 36 gr Blanc </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 36 gr Clair Rebut </t>
+  </si>
+  <si>
+    <t>Préformes 23gr Bleu GMAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 23 gr Blanc </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 16 gr Clair </t>
+  </si>
+  <si>
+    <t>HDPE Blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDPE Vert </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDPE Mélange </t>
+  </si>
+  <si>
+    <t>HDPE Jaune</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDPE Orange </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDPE Rose </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDPE Marron </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDPE Bleu </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PET Broyé </t>
+  </si>
+  <si>
+    <t>Matière Broyée Blanc</t>
+  </si>
+  <si>
+    <t>Matière Broyée Vert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Rouge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Jaune </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Noire </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Orange </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Violet </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Claire </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Bleu </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyée Mélange </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masterbatch Blanc </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masterbatch Vert </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masterbatch Rouge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masterbatch Jaune </t>
+  </si>
+  <si>
+    <t>Masterbatch Noir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masterbatch Violet </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masterbatch Bleu </t>
+  </si>
+  <si>
+    <t>Préformes 19 gr TOSHIBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière broyé Vierge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière broyé Marron </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Après convoyeur </t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 gr Husky Avec Additif </t>
+  </si>
+  <si>
+    <t>Préforme 27,5 gr Clair</t>
+  </si>
+  <si>
+    <t>Préformes 22,5 gr Clair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anse de Sceau </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préformes 24 Gr </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière Broyé Fushia </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Broyer Vert Foncé </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cageot </t>
+  </si>
+  <si>
+    <t>Masterbatch bleu marine</t>
+  </si>
+  <si>
+    <t>Masterbatch fuschia</t>
+  </si>
+  <si>
+    <t>Broyer bidon rouge</t>
+  </si>
+  <si>
+    <t>Glacière blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préforme 20 gr Marron </t>
+  </si>
+  <si>
+    <t>Broyer fushia</t>
+  </si>
+  <si>
+    <t>Broyer grenat</t>
+  </si>
+  <si>
+    <t>cône</t>
+  </si>
+  <si>
+    <t>Bouchon Rouge</t>
+  </si>
+  <si>
+    <t>Bouchon Bleu</t>
+  </si>
+  <si>
+    <t>Bouchon Vert</t>
+  </si>
+  <si>
+    <t>bidon blanc somapro</t>
+  </si>
+  <si>
+    <t>broyer gris</t>
+  </si>
+  <si>
+    <t>bouchons mélange</t>
+  </si>
+  <si>
+    <t>Matière broyé beige</t>
+  </si>
+  <si>
+    <t>bouchon blanc</t>
+  </si>
+  <si>
+    <t>yop</t>
+  </si>
+  <si>
+    <t>bouchon jaune</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préforme 19 gr IMRA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cône mélange </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bouteille HDPE </t>
+  </si>
+  <si>
+    <t>matiere</t>
   </si>
 </sst>
 </file>
@@ -687,7 +901,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -695,7 +909,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.75" customWidth="1"/>
@@ -2426,6 +2640,3141 @@
         <v>392</v>
       </c>
     </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="1"/>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="1"/>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" s="1"/>
+    </row>
+    <row r="90" spans="1:6">
+      <c r="A90" s="1"/>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" s="1"/>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" s="1"/>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" s="1"/>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="1"/>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" s="1"/>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" s="1"/>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" s="1"/>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" s="1"/>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" s="1"/>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" s="1"/>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" s="1"/>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" s="1"/>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" s="1"/>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" s="1"/>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="1"/>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" s="1"/>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" s="1"/>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" s="1"/>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" s="1"/>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" s="1"/>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" s="1"/>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" s="1"/>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" s="1"/>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" s="1"/>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" s="1"/>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" s="1"/>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" s="1"/>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" s="1"/>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" s="1"/>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" s="1"/>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" s="1"/>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" s="1"/>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123" s="1"/>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" s="1"/>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125" s="1"/>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" s="1"/>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127" s="1"/>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" s="1"/>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129" s="1"/>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" s="1"/>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" s="1"/>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" s="1"/>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" s="1"/>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" s="1"/>
+    </row>
+    <row r="135" spans="1:1">
+      <c r="A135" s="1"/>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136" s="1"/>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137" s="1"/>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" s="1"/>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139" s="1"/>
+    </row>
+    <row r="140" spans="1:1">
+      <c r="A140" s="1"/>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141" s="1"/>
+    </row>
+    <row r="142" spans="1:1">
+      <c r="A142" s="1"/>
+    </row>
+    <row r="143" spans="1:1">
+      <c r="A143" s="1"/>
+    </row>
+    <row r="144" spans="1:1">
+      <c r="A144" s="1"/>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" s="1"/>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" s="1"/>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147" s="1"/>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148" s="1"/>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" s="1"/>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" s="1"/>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" s="1"/>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" s="1"/>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" s="1"/>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" s="1"/>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" s="1"/>
+    </row>
+    <row r="156" spans="1:1">
+      <c r="A156" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F156"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="11.75" customWidth="1"/>
+    <col min="2" max="2" width="11.125" customWidth="1"/>
+    <col min="3" max="3" width="31" style="2" customWidth="1"/>
+    <col min="4" max="4" width="26" style="3" customWidth="1"/>
+    <col min="5" max="5" width="6.625" customWidth="1"/>
+    <col min="6" max="6" width="11.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>7746</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>4329</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2">
+        <v>5</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="1">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="1">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>2730</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="1">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="1">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2">
+        <v>9</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>4428</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="1">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2">
+        <v>10</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="1">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2">
+        <v>11</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>7298</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="1">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2">
+        <v>12</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="1">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2">
+        <v>13</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="1">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2">
+        <v>14</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="1">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="2">
+        <v>15</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="1">
+        <v>2</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2">
+        <v>16</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="1">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2">
+        <v>17</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="1">
+        <v>2</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="2">
+        <v>18</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="1">
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2">
+        <v>19</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="1">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="2">
+        <v>20</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="1">
+        <v>2</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="2">
+        <v>21</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="1">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="2">
+        <v>22</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="1">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="2">
+        <v>23</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>2765</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="1">
+        <v>2</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="2">
+        <v>24</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="1">
+        <v>2</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="2">
+        <v>25</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="1">
+        <v>2</v>
+      </c>
+      <c r="B27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="2">
+        <v>26</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="1">
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="2">
+        <v>27</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="1">
+        <v>2</v>
+      </c>
+      <c r="B29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="2">
+        <v>28</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="1">
+        <v>2</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="2">
+        <v>29</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="1">
+        <v>2</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="2">
+        <v>30</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="1">
+        <v>2</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="2">
+        <v>31</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="1">
+        <v>2</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="2">
+        <v>32</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="1">
+        <v>2</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="2">
+        <v>33</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="1">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="2">
+        <v>34</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="1">
+        <v>2</v>
+      </c>
+      <c r="B36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="2">
+        <v>35</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="1">
+        <v>2</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="2">
+        <v>36</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="1">
+        <v>2</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="2">
+        <v>37</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="1">
+        <v>2</v>
+      </c>
+      <c r="B39" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="2">
+        <v>38</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="1">
+        <v>2</v>
+      </c>
+      <c r="B40" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="2">
+        <v>39</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="1">
+        <v>2</v>
+      </c>
+      <c r="B41" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="2">
+        <v>40</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="1">
+        <v>2</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="2">
+        <v>41</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="1">
+        <v>2</v>
+      </c>
+      <c r="B43" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="2">
+        <v>42</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="1">
+        <v>2</v>
+      </c>
+      <c r="B44" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="2">
+        <v>43</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="F44">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="1">
+        <v>2</v>
+      </c>
+      <c r="B45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="2">
+        <v>44</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="1">
+        <v>2</v>
+      </c>
+      <c r="B46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="2">
+        <v>45</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="1">
+        <v>2</v>
+      </c>
+      <c r="B47" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="2">
+        <v>46</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="1">
+        <v>2</v>
+      </c>
+      <c r="B48" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="2">
+        <v>47</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <v>16266</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="1">
+        <v>2</v>
+      </c>
+      <c r="B49" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="2">
+        <v>48</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="1">
+        <v>2</v>
+      </c>
+      <c r="B50" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="2">
+        <v>49</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="1">
+        <v>2</v>
+      </c>
+      <c r="B51" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="2">
+        <v>50</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="1">
+        <v>2</v>
+      </c>
+      <c r="B52" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="2">
+        <v>51</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="1">
+        <v>2</v>
+      </c>
+      <c r="B53" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="2">
+        <v>52</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="1">
+        <v>2</v>
+      </c>
+      <c r="B54" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="2">
+        <v>53</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="1">
+        <v>2</v>
+      </c>
+      <c r="B55" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="2">
+        <v>54</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="1">
+        <v>2</v>
+      </c>
+      <c r="B56" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" s="2">
+        <v>55</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="1">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="2">
+        <v>56</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
+      </c>
+      <c r="F57">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="1">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="2">
+        <v>57</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="F58">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="1">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="2">
+        <v>58</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="1">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="2">
+        <v>59</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E60">
+        <v>1</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="1">
+        <v>2</v>
+      </c>
+      <c r="B61" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="2">
+        <v>60</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E61">
+        <v>1</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" s="1">
+        <v>2</v>
+      </c>
+      <c r="B62" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="2">
+        <v>61</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+      <c r="F62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="1">
+        <v>2</v>
+      </c>
+      <c r="B63" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="2">
+        <v>62</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E63">
+        <v>1</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="1">
+        <v>2</v>
+      </c>
+      <c r="B64" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="2">
+        <v>63</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E64">
+        <v>1</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="1">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="2">
+        <v>64</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E65">
+        <v>1</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" s="1">
+        <v>2</v>
+      </c>
+      <c r="B66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" s="2">
+        <v>65</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" s="1">
+        <v>2</v>
+      </c>
+      <c r="B67" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="2">
+        <v>66</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E67">
+        <v>1</v>
+      </c>
+      <c r="F67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" s="1">
+        <v>2</v>
+      </c>
+      <c r="B68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="2">
+        <v>67</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E68">
+        <v>1</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" s="1">
+        <v>2</v>
+      </c>
+      <c r="B69" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="2">
+        <v>68</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E69">
+        <v>1</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" s="1">
+        <v>2</v>
+      </c>
+      <c r="B70" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="2">
+        <v>69</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E70">
+        <v>1</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" s="1">
+        <v>2</v>
+      </c>
+      <c r="B71" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="2">
+        <v>70</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E71">
+        <v>1</v>
+      </c>
+      <c r="F71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="1">
+        <v>2</v>
+      </c>
+      <c r="B72" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="2">
+        <v>71</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E72">
+        <v>1</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="1">
+        <v>2</v>
+      </c>
+      <c r="B73" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="2">
+        <v>72</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
+      <c r="F73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" s="1">
+        <v>2</v>
+      </c>
+      <c r="B74" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" s="2">
+        <v>73</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E74">
+        <v>1</v>
+      </c>
+      <c r="F74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" s="1">
+        <v>2</v>
+      </c>
+      <c r="B75" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="2">
+        <v>74</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E75">
+        <v>1</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="1">
+        <v>2</v>
+      </c>
+      <c r="B76" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="2">
+        <v>75</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E76">
+        <v>1</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" s="1">
+        <v>2</v>
+      </c>
+      <c r="B77" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="2">
+        <v>76</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E77">
+        <v>1</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" s="1">
+        <v>2</v>
+      </c>
+      <c r="B78" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="2">
+        <v>77</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" s="1">
+        <v>2</v>
+      </c>
+      <c r="B79" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="2">
+        <v>78</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E79">
+        <v>1</v>
+      </c>
+      <c r="F79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" s="1">
+        <v>2</v>
+      </c>
+      <c r="B80" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" s="2">
+        <v>79</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E80">
+        <v>1</v>
+      </c>
+      <c r="F80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
+      <c r="A81" s="1">
+        <v>2</v>
+      </c>
+      <c r="B81" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="2">
+        <v>80</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
+      <c r="A82" s="1">
+        <v>2</v>
+      </c>
+      <c r="B82" t="s">
+        <v>4</v>
+      </c>
+      <c r="C82" s="2">
+        <v>81</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E82">
+        <v>1</v>
+      </c>
+      <c r="F82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
+      <c r="A83" s="1">
+        <v>2</v>
+      </c>
+      <c r="B83" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" s="2">
+        <v>82</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
+      <c r="F83">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" s="1">
+        <v>2</v>
+      </c>
+      <c r="B84" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" s="2">
+        <v>83</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
+      <c r="A85" s="1">
+        <v>2</v>
+      </c>
+      <c r="B85" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="2">
+        <v>84</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85">
+        <v>5238</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" s="1">
+        <v>2</v>
+      </c>
+      <c r="B86" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" s="2">
+        <v>85</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="1">
+        <v>2</v>
+      </c>
+      <c r="B87" t="s">
+        <v>162</v>
+      </c>
+      <c r="C87" s="2">
+        <v>86</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="1">
+        <v>2</v>
+      </c>
+      <c r="B88" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" s="2">
+        <v>87</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" s="1">
+        <v>2</v>
+      </c>
+      <c r="B89" t="s">
+        <v>162</v>
+      </c>
+      <c r="C89" s="2">
+        <v>88</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F89">
+        <v>74799</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6">
+      <c r="A90" s="1">
+        <v>2</v>
+      </c>
+      <c r="B90" t="s">
+        <v>162</v>
+      </c>
+      <c r="C90" s="2">
+        <v>89</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" s="1">
+        <v>2</v>
+      </c>
+      <c r="B91" t="s">
+        <v>162</v>
+      </c>
+      <c r="C91" s="2">
+        <v>90</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F91">
+        <v>69410</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" s="1">
+        <v>2</v>
+      </c>
+      <c r="B92" t="s">
+        <v>162</v>
+      </c>
+      <c r="C92" s="2">
+        <v>91</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" s="1">
+        <v>2</v>
+      </c>
+      <c r="B93" t="s">
+        <v>162</v>
+      </c>
+      <c r="C93" s="2">
+        <v>92</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="1">
+        <v>2</v>
+      </c>
+      <c r="B94" t="s">
+        <v>162</v>
+      </c>
+      <c r="C94" s="2">
+        <v>93</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" s="1">
+        <v>2</v>
+      </c>
+      <c r="B95" t="s">
+        <v>162</v>
+      </c>
+      <c r="C95" s="2">
+        <v>94</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" s="1">
+        <v>2</v>
+      </c>
+      <c r="B96" t="s">
+        <v>162</v>
+      </c>
+      <c r="C96" s="2">
+        <v>95</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
+      <c r="A97" s="1">
+        <v>2</v>
+      </c>
+      <c r="B97" t="s">
+        <v>162</v>
+      </c>
+      <c r="C97" s="2">
+        <v>96</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F97">
+        <v>-4705</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6">
+      <c r="A98" s="1">
+        <v>2</v>
+      </c>
+      <c r="B98" t="s">
+        <v>162</v>
+      </c>
+      <c r="C98" s="2">
+        <v>97</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F98">
+        <v>1475.0000000000018</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
+      <c r="A99" s="1">
+        <v>2</v>
+      </c>
+      <c r="B99" t="s">
+        <v>162</v>
+      </c>
+      <c r="C99" s="2">
+        <v>98</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6">
+      <c r="A100" s="1">
+        <v>2</v>
+      </c>
+      <c r="B100" t="s">
+        <v>162</v>
+      </c>
+      <c r="C100" s="2">
+        <v>99</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6">
+      <c r="A101" s="1">
+        <v>2</v>
+      </c>
+      <c r="B101" t="s">
+        <v>162</v>
+      </c>
+      <c r="C101" s="2">
+        <v>100</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6">
+      <c r="A102" s="1">
+        <v>2</v>
+      </c>
+      <c r="B102" t="s">
+        <v>162</v>
+      </c>
+      <c r="C102" s="2">
+        <v>101</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6">
+      <c r="A103" s="1">
+        <v>2</v>
+      </c>
+      <c r="B103" t="s">
+        <v>162</v>
+      </c>
+      <c r="C103" s="2">
+        <v>102</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
+      <c r="A104" s="1">
+        <v>2</v>
+      </c>
+      <c r="B104" t="s">
+        <v>162</v>
+      </c>
+      <c r="C104" s="2">
+        <v>103</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
+      <c r="A105" s="1">
+        <v>2</v>
+      </c>
+      <c r="B105" t="s">
+        <v>162</v>
+      </c>
+      <c r="C105" s="2">
+        <v>104</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6">
+      <c r="A106" s="1">
+        <v>2</v>
+      </c>
+      <c r="B106" t="s">
+        <v>162</v>
+      </c>
+      <c r="C106" s="2">
+        <v>105</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6">
+      <c r="A107" s="1">
+        <v>2</v>
+      </c>
+      <c r="B107" t="s">
+        <v>162</v>
+      </c>
+      <c r="C107" s="2">
+        <v>106</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F107">
+        <v>3291.1700000000019</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6">
+      <c r="A108" s="1">
+        <v>2</v>
+      </c>
+      <c r="B108" t="s">
+        <v>162</v>
+      </c>
+      <c r="C108" s="2">
+        <v>107</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F108">
+        <v>62.480000000001382</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6">
+      <c r="A109" s="1">
+        <v>2</v>
+      </c>
+      <c r="B109" t="s">
+        <v>162</v>
+      </c>
+      <c r="C109" s="2">
+        <v>108</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F109">
+        <v>90.119999999999891</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6">
+      <c r="A110" s="1">
+        <v>2</v>
+      </c>
+      <c r="B110" t="s">
+        <v>162</v>
+      </c>
+      <c r="C110" s="2">
+        <v>109</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F110">
+        <v>439.64000000000306</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
+      <c r="A111" s="1">
+        <v>2</v>
+      </c>
+      <c r="B111" t="s">
+        <v>162</v>
+      </c>
+      <c r="C111" s="2">
+        <v>110</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F111">
+        <v>121.34</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6">
+      <c r="A112" s="1">
+        <v>2</v>
+      </c>
+      <c r="B112" t="s">
+        <v>162</v>
+      </c>
+      <c r="C112" s="2">
+        <v>111</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F112">
+        <v>92.050000000000182</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6">
+      <c r="A113" s="1">
+        <v>2</v>
+      </c>
+      <c r="B113" t="s">
+        <v>162</v>
+      </c>
+      <c r="C113" s="2">
+        <v>112</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F113">
+        <v>149.38999999999942</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6">
+      <c r="A114" s="1">
+        <v>2</v>
+      </c>
+      <c r="B114" t="s">
+        <v>162</v>
+      </c>
+      <c r="C114" s="2">
+        <v>113</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6">
+      <c r="A115" s="1">
+        <v>2</v>
+      </c>
+      <c r="B115" t="s">
+        <v>162</v>
+      </c>
+      <c r="C115" s="2">
+        <v>114</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F115">
+        <v>2013.1410000000033</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6">
+      <c r="A116" s="1">
+        <v>2</v>
+      </c>
+      <c r="B116" t="s">
+        <v>162</v>
+      </c>
+      <c r="C116" s="2">
+        <v>115</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F116">
+        <v>18.060000000000059</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6">
+      <c r="A117" s="1">
+        <v>2</v>
+      </c>
+      <c r="B117" t="s">
+        <v>162</v>
+      </c>
+      <c r="C117" s="2">
+        <v>116</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F117">
+        <v>2.5999999999999996</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6">
+      <c r="A118" s="1">
+        <v>2</v>
+      </c>
+      <c r="B118" t="s">
+        <v>162</v>
+      </c>
+      <c r="C118" s="2">
+        <v>117</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F118">
+        <v>17.512999999999998</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="A119" s="1">
+        <v>2</v>
+      </c>
+      <c r="B119" t="s">
+        <v>162</v>
+      </c>
+      <c r="C119" s="2">
+        <v>118</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="F119">
+        <v>41.523200000000003</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
+      <c r="A120" s="1">
+        <v>2</v>
+      </c>
+      <c r="B120" t="s">
+        <v>162</v>
+      </c>
+      <c r="C120" s="2">
+        <v>119</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F120">
+        <v>16.992800000000006</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6">
+      <c r="A121" s="1">
+        <v>2</v>
+      </c>
+      <c r="B121" t="s">
+        <v>162</v>
+      </c>
+      <c r="C121" s="2">
+        <v>120</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F121">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6">
+      <c r="A122" s="1">
+        <v>2</v>
+      </c>
+      <c r="B122" t="s">
+        <v>162</v>
+      </c>
+      <c r="C122" s="2">
+        <v>121</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="F122">
+        <v>9.9990000000000023</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6">
+      <c r="A123" s="1">
+        <v>2</v>
+      </c>
+      <c r="B123" t="s">
+        <v>162</v>
+      </c>
+      <c r="C123" s="2">
+        <v>122</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F123">
+        <v>20.891999999999996</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6">
+      <c r="A124" s="1">
+        <v>2</v>
+      </c>
+      <c r="B124" t="s">
+        <v>162</v>
+      </c>
+      <c r="C124" s="2">
+        <v>123</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="F124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6">
+      <c r="A125" s="1">
+        <v>2</v>
+      </c>
+      <c r="B125" t="s">
+        <v>162</v>
+      </c>
+      <c r="C125" s="2">
+        <v>124</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="F125">
+        <v>563.25000000000455</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6">
+      <c r="A126" s="1">
+        <v>2</v>
+      </c>
+      <c r="B126" t="s">
+        <v>162</v>
+      </c>
+      <c r="C126" s="2">
+        <v>125</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F126">
+        <v>197.68</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6">
+      <c r="A127" s="1">
+        <v>2</v>
+      </c>
+      <c r="B127" t="s">
+        <v>162</v>
+      </c>
+      <c r="C127" s="2">
+        <v>126</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="F127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6">
+      <c r="A128" s="1">
+        <v>2</v>
+      </c>
+      <c r="B128" t="s">
+        <v>162</v>
+      </c>
+      <c r="C128" s="2">
+        <v>127</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F128">
+        <v>54753</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6">
+      <c r="A129" s="1">
+        <v>2</v>
+      </c>
+      <c r="B129" t="s">
+        <v>162</v>
+      </c>
+      <c r="C129" s="2">
+        <v>128</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6">
+      <c r="A130" s="1">
+        <v>2</v>
+      </c>
+      <c r="B130" t="s">
+        <v>162</v>
+      </c>
+      <c r="C130" s="2">
+        <v>129</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F130">
+        <v>-563</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6">
+      <c r="A131" s="1">
+        <v>2</v>
+      </c>
+      <c r="B131" t="s">
+        <v>162</v>
+      </c>
+      <c r="C131" s="2">
+        <v>130</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="F131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6">
+      <c r="A132" s="1">
+        <v>2</v>
+      </c>
+      <c r="B132" t="s">
+        <v>162</v>
+      </c>
+      <c r="C132" s="2">
+        <v>131</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6">
+      <c r="A133" s="1">
+        <v>2</v>
+      </c>
+      <c r="B133" t="s">
+        <v>162</v>
+      </c>
+      <c r="C133" s="2">
+        <v>132</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6">
+      <c r="A134" s="1">
+        <v>2</v>
+      </c>
+      <c r="B134" t="s">
+        <v>162</v>
+      </c>
+      <c r="C134" s="2">
+        <v>133</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6">
+      <c r="A135" s="1">
+        <v>2</v>
+      </c>
+      <c r="B135" t="s">
+        <v>162</v>
+      </c>
+      <c r="C135" s="2">
+        <v>134</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="F135">
+        <v>2096.75</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6">
+      <c r="A136" s="1">
+        <v>2</v>
+      </c>
+      <c r="B136" t="s">
+        <v>162</v>
+      </c>
+      <c r="C136" s="2">
+        <v>135</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="F136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6">
+      <c r="A137" s="1">
+        <v>2</v>
+      </c>
+      <c r="B137" t="s">
+        <v>162</v>
+      </c>
+      <c r="C137" s="2">
+        <v>136</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F137">
+        <v>15.472999999999999</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6">
+      <c r="A138" s="1">
+        <v>2</v>
+      </c>
+      <c r="B138" t="s">
+        <v>162</v>
+      </c>
+      <c r="C138" s="2">
+        <v>137</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6">
+      <c r="A139" s="1">
+        <v>2</v>
+      </c>
+      <c r="B139" t="s">
+        <v>162</v>
+      </c>
+      <c r="C139" s="2">
+        <v>138</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="F139">
+        <v>-5.6843418860808015E-14</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6">
+      <c r="A140" s="1">
+        <v>2</v>
+      </c>
+      <c r="B140" t="s">
+        <v>162</v>
+      </c>
+      <c r="C140" s="2">
+        <v>139</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F140">
+        <v>-4333</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6">
+      <c r="A141" s="1">
+        <v>2</v>
+      </c>
+      <c r="B141" t="s">
+        <v>162</v>
+      </c>
+      <c r="C141" s="2">
+        <v>140</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F141">
+        <v>-2.8421709430404007E-14</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6">
+      <c r="A142" s="1">
+        <v>2</v>
+      </c>
+      <c r="B142" t="s">
+        <v>162</v>
+      </c>
+      <c r="C142" s="2">
+        <v>141</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6">
+      <c r="A143" s="1">
+        <v>2</v>
+      </c>
+      <c r="B143" t="s">
+        <v>162</v>
+      </c>
+      <c r="C143" s="2">
+        <v>142</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6">
+      <c r="A144" s="1">
+        <v>2</v>
+      </c>
+      <c r="B144" t="s">
+        <v>162</v>
+      </c>
+      <c r="C144" s="2">
+        <v>143</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6">
+      <c r="A145" s="1">
+        <v>2</v>
+      </c>
+      <c r="B145" t="s">
+        <v>162</v>
+      </c>
+      <c r="C145" s="2">
+        <v>144</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6">
+      <c r="A146" s="1">
+        <v>2</v>
+      </c>
+      <c r="B146" t="s">
+        <v>162</v>
+      </c>
+      <c r="C146" s="2">
+        <v>145</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6">
+      <c r="A147" s="1">
+        <v>2</v>
+      </c>
+      <c r="B147" t="s">
+        <v>162</v>
+      </c>
+      <c r="C147" s="2">
+        <v>146</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6">
+      <c r="A148" s="1">
+        <v>2</v>
+      </c>
+      <c r="B148" t="s">
+        <v>162</v>
+      </c>
+      <c r="C148" s="2">
+        <v>147</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F148">
+        <v>37.459999999999923</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6">
+      <c r="A149" s="1">
+        <v>2</v>
+      </c>
+      <c r="B149" t="s">
+        <v>162</v>
+      </c>
+      <c r="C149" s="2">
+        <v>148</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F149">
+        <v>37.679999999999993</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6">
+      <c r="A150" s="1">
+        <v>2</v>
+      </c>
+      <c r="B150" t="s">
+        <v>162</v>
+      </c>
+      <c r="C150" s="2">
+        <v>149</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F150">
+        <v>-235.48000000000002</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6">
+      <c r="A151" s="1">
+        <v>2</v>
+      </c>
+      <c r="B151" t="s">
+        <v>162</v>
+      </c>
+      <c r="C151" s="2">
+        <v>150</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="F151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6">
+      <c r="A152" s="1">
+        <v>2</v>
+      </c>
+      <c r="B152" t="s">
+        <v>162</v>
+      </c>
+      <c r="C152" s="2">
+        <v>151</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F152">
+        <v>235.48</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6">
+      <c r="A153" s="1">
+        <v>2</v>
+      </c>
+      <c r="B153" t="s">
+        <v>162</v>
+      </c>
+      <c r="C153" s="2">
+        <v>152</v>
+      </c>
+      <c r="D153" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6">
+      <c r="A154" s="1">
+        <v>2</v>
+      </c>
+      <c r="B154" t="s">
+        <v>162</v>
+      </c>
+      <c r="C154" s="2">
+        <v>153</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6">
+      <c r="A155" s="1">
+        <v>2</v>
+      </c>
+      <c r="B155" t="s">
+        <v>162</v>
+      </c>
+      <c r="C155" s="2">
+        <v>154</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="F155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6">
+      <c r="A156" s="1">
+        <v>2</v>
+      </c>
+      <c r="B156" t="s">
+        <v>162</v>
+      </c>
+      <c r="C156" s="2">
+        <v>155</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F156">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Module Reports and dashboard + exports
</commit_message>
<xml_diff>
--- a/backend-erp/database/seeders/data/Stocks.xlsx
+++ b/backend-erp/database/seeders/data/Stocks.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="146">
   <si>
     <t>location_id</t>
   </si>
@@ -312,150 +312,33 @@
     <t>Bouchon HDPE Fanta Orange</t>
   </si>
   <si>
-    <t xml:space="preserve">Préformes 19 gr Clair Dmag </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 19gr Clair Husky </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 19 gr Blanc </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 36gr Husky </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 36 gr Toshiba </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 36 gr Blanc </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 36 gr Clair Rebut </t>
-  </si>
-  <si>
     <t>Préformes 23gr Bleu GMAG</t>
   </si>
   <si>
-    <t xml:space="preserve">Préformes 23 gr Blanc </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 16 gr Clair </t>
-  </si>
-  <si>
     <t>HDPE Blanc</t>
   </si>
   <si>
-    <t xml:space="preserve">HDPE Vert </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDPE Mélange </t>
-  </si>
-  <si>
     <t>HDPE Jaune</t>
   </si>
   <si>
-    <t xml:space="preserve">HDPE Orange </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDPE Rose </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDPE Marron </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDPE Bleu </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PET Broyé </t>
-  </si>
-  <si>
     <t>Matière Broyée Blanc</t>
   </si>
   <si>
     <t>Matière Broyée Vert</t>
   </si>
   <si>
-    <t xml:space="preserve">Matière Broyée Rouge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyée Jaune </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyée Noire </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyée Orange </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyée Violet </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyée Claire </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyée Bleu </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyée Mélange </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masterbatch Blanc </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masterbatch Vert </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masterbatch Rouge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masterbatch Jaune </t>
-  </si>
-  <si>
     <t>Masterbatch Noir</t>
   </si>
   <si>
-    <t xml:space="preserve">Masterbatch Violet </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masterbatch Bleu </t>
-  </si>
-  <si>
     <t>Préformes 19 gr TOSHIBA</t>
   </si>
   <si>
-    <t xml:space="preserve">Matière broyé Vierge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière broyé Marron </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Après convoyeur </t>
-  </si>
-  <si>
-    <t xml:space="preserve">19 gr Husky Avec Additif </t>
-  </si>
-  <si>
     <t>Préforme 27,5 gr Clair</t>
   </si>
   <si>
     <t>Préformes 22,5 gr Clair</t>
   </si>
   <si>
-    <t xml:space="preserve">Anse de Sceau </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préformes 24 Gr </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matière Broyé Fushia </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broyer Vert Foncé </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Cageot </t>
-  </si>
-  <si>
     <t>Masterbatch bleu marine</t>
   </si>
   <si>
@@ -468,58 +351,124 @@
     <t>Glacière blanc</t>
   </si>
   <si>
-    <t xml:space="preserve">Préforme 20 gr Marron </t>
-  </si>
-  <si>
-    <t>Broyer fushia</t>
-  </si>
-  <si>
-    <t>Broyer grenat</t>
-  </si>
-  <si>
-    <t>cône</t>
-  </si>
-  <si>
-    <t>Bouchon Rouge</t>
-  </si>
-  <si>
-    <t>Bouchon Bleu</t>
-  </si>
-  <si>
-    <t>Bouchon Vert</t>
-  </si>
-  <si>
-    <t>bidon blanc somapro</t>
-  </si>
-  <si>
-    <t>broyer gris</t>
-  </si>
-  <si>
-    <t>bouchons mélange</t>
-  </si>
-  <si>
-    <t>Matière broyé beige</t>
-  </si>
-  <si>
-    <t>bouchon blanc</t>
-  </si>
-  <si>
-    <t>yop</t>
-  </si>
-  <si>
-    <t>bouchon jaune</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préforme 19 gr IMRA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cône mélange </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bouteille HDPE </t>
-  </si>
-  <si>
     <t>matiere</t>
+  </si>
+  <si>
+    <t>Préformes 19 gr Clair Dmag</t>
+  </si>
+  <si>
+    <t>Préformes 19gr Clair Husky</t>
+  </si>
+  <si>
+    <t>Préformes 19 gr Blanc</t>
+  </si>
+  <si>
+    <t>Préformes 36gr Husky</t>
+  </si>
+  <si>
+    <t>Préformes 36 gr Toshiba</t>
+  </si>
+  <si>
+    <t>Préformes 36 gr Blanc</t>
+  </si>
+  <si>
+    <t>Préformes 36 gr Clair Rebut</t>
+  </si>
+  <si>
+    <t>Préformes 23 gr Blanc</t>
+  </si>
+  <si>
+    <t>Préformes 16 gr Clair</t>
+  </si>
+  <si>
+    <t>HDPE Vert</t>
+  </si>
+  <si>
+    <t>HDPE Mélange</t>
+  </si>
+  <si>
+    <t>HDPE Orange</t>
+  </si>
+  <si>
+    <t>HDPE Rose</t>
+  </si>
+  <si>
+    <t>HDPE Marron</t>
+  </si>
+  <si>
+    <t>HDPE Bleu</t>
+  </si>
+  <si>
+    <t>PET Broyé</t>
+  </si>
+  <si>
+    <t>Matière Broyée Rouge</t>
+  </si>
+  <si>
+    <t>Matière Broyée Jaune</t>
+  </si>
+  <si>
+    <t>Matière Broyée Noire</t>
+  </si>
+  <si>
+    <t>Matière Broyée Orange</t>
+  </si>
+  <si>
+    <t>Matière Broyée Violet</t>
+  </si>
+  <si>
+    <t>Matière Broyée Claire</t>
+  </si>
+  <si>
+    <t>Matière Broyée Bleu</t>
+  </si>
+  <si>
+    <t>Matière Broyée Mélange</t>
+  </si>
+  <si>
+    <t>Masterbatch Blanc</t>
+  </si>
+  <si>
+    <t>Masterbatch Vert</t>
+  </si>
+  <si>
+    <t>Masterbatch Rouge</t>
+  </si>
+  <si>
+    <t>Masterbatch Jaune</t>
+  </si>
+  <si>
+    <t>Masterbatch Violet</t>
+  </si>
+  <si>
+    <t>Masterbatch Bleu</t>
+  </si>
+  <si>
+    <t>Matière broyé Vierge</t>
+  </si>
+  <si>
+    <t>Matière broyé Marron</t>
+  </si>
+  <si>
+    <t>Après convoyeur</t>
+  </si>
+  <si>
+    <t>19 gr Husky Avec Additif</t>
+  </si>
+  <si>
+    <t>Anse de Sceau</t>
+  </si>
+  <si>
+    <t>Préformes 24 Gr</t>
+  </si>
+  <si>
+    <t>Matière Broyé Fushia</t>
+  </si>
+  <si>
+    <t>Broyer Vert Foncé</t>
+  </si>
+  <si>
+    <t>Préforme 20 gr Marron</t>
   </si>
 </sst>
 </file>
@@ -901,7 +850,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2857,7 +2806,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F156"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.75" customWidth="1"/>
@@ -4593,7 +4542,7 @@
         <v>2</v>
       </c>
       <c r="B87" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C87" s="2">
         <v>86</v>
@@ -4602,7 +4551,7 @@
         <v>92</v>
       </c>
       <c r="F87">
-        <v>0</v>
+        <v>3189</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -4610,13 +4559,13 @@
         <v>2</v>
       </c>
       <c r="B88" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C88" s="2">
         <v>87</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="F88">
         <v>0</v>
@@ -4627,16 +4576,16 @@
         <v>2</v>
       </c>
       <c r="B89" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C89" s="2">
         <v>88</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="F89">
-        <v>74799</v>
+        <v>35539</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -4644,13 +4593,13 @@
         <v>2</v>
       </c>
       <c r="B90" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C90" s="2">
         <v>89</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="F90">
         <v>0</v>
@@ -4661,16 +4610,16 @@
         <v>2</v>
       </c>
       <c r="B91" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C91" s="2">
         <v>90</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="F91">
-        <v>69410</v>
+        <v>35814</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -4678,13 +4627,13 @@
         <v>2</v>
       </c>
       <c r="B92" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C92" s="2">
         <v>91</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="F92">
         <v>0</v>
@@ -4695,13 +4644,13 @@
         <v>2</v>
       </c>
       <c r="B93" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C93" s="2">
         <v>92</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="F93">
         <v>0</v>
@@ -4712,13 +4661,13 @@
         <v>2</v>
       </c>
       <c r="B94" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C94" s="2">
         <v>93</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="F94">
         <v>0</v>
@@ -4729,16 +4678,16 @@
         <v>2</v>
       </c>
       <c r="B95" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C95" s="2">
         <v>94</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F95">
-        <v>0</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -4746,13 +4695,13 @@
         <v>2</v>
       </c>
       <c r="B96" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C96" s="2">
         <v>95</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -4760,16 +4709,16 @@
         <v>2</v>
       </c>
       <c r="B97" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C97" s="2">
         <v>96</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="F97">
-        <v>-4705</v>
+        <v>56001</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -4777,16 +4726,16 @@
         <v>2</v>
       </c>
       <c r="B98" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C98" s="2">
         <v>97</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="F98">
-        <v>1475.0000000000018</v>
+        <v>126.6899999999996</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -4794,13 +4743,13 @@
         <v>2</v>
       </c>
       <c r="B99" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C99" s="2">
         <v>98</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="F99">
         <v>0</v>
@@ -4811,13 +4760,13 @@
         <v>2</v>
       </c>
       <c r="B100" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C100" s="2">
         <v>99</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="F100">
         <v>0</v>
@@ -4828,13 +4777,13 @@
         <v>2</v>
       </c>
       <c r="B101" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C101" s="2">
         <v>100</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="F101">
         <v>0</v>
@@ -4845,13 +4794,13 @@
         <v>2</v>
       </c>
       <c r="B102" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C102" s="2">
         <v>101</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="F102">
         <v>0</v>
@@ -4862,13 +4811,13 @@
         <v>2</v>
       </c>
       <c r="B103" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C103" s="2">
         <v>102</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="F103">
         <v>0</v>
@@ -4879,13 +4828,13 @@
         <v>2</v>
       </c>
       <c r="B104" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C104" s="2">
         <v>103</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="F104">
         <v>0</v>
@@ -4896,13 +4845,13 @@
         <v>2</v>
       </c>
       <c r="B105" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C105" s="2">
         <v>104</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="F105">
         <v>0</v>
@@ -4913,16 +4862,16 @@
         <v>2</v>
       </c>
       <c r="B106" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C106" s="2">
         <v>105</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="F106">
-        <v>0</v>
+        <v>1892.38</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -4930,16 +4879,16 @@
         <v>2</v>
       </c>
       <c r="B107" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C107" s="2">
         <v>106</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="F107">
-        <v>3291.1700000000019</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -4947,16 +4896,16 @@
         <v>2</v>
       </c>
       <c r="B108" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C108" s="2">
         <v>107</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="F108">
-        <v>62.480000000001382</v>
+        <v>161.43999999999983</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -4964,16 +4913,16 @@
         <v>2</v>
       </c>
       <c r="B109" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C109" s="2">
         <v>108</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F109">
-        <v>90.119999999999891</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -4981,16 +4930,16 @@
         <v>2</v>
       </c>
       <c r="B110" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C110" s="2">
         <v>109</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="F110">
-        <v>439.64000000000306</v>
+        <v>171.29999999999995</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -4998,16 +4947,16 @@
         <v>2</v>
       </c>
       <c r="B111" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C111" s="2">
         <v>110</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="F111">
-        <v>121.34</v>
+        <v>49.02</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -5015,16 +4964,16 @@
         <v>2</v>
       </c>
       <c r="B112" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C112" s="2">
         <v>111</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="F112">
-        <v>92.050000000000182</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -5032,16 +4981,16 @@
         <v>2</v>
       </c>
       <c r="B113" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C113" s="2">
         <v>112</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="F113">
-        <v>149.38999999999942</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -5049,16 +4998,16 @@
         <v>2</v>
       </c>
       <c r="B114" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C114" s="2">
         <v>113</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="F114">
-        <v>0</v>
+        <v>48.82</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -5066,16 +5015,16 @@
         <v>2</v>
       </c>
       <c r="B115" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C115" s="2">
         <v>114</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="F115">
-        <v>2013.1410000000033</v>
+        <v>23.550999999999931</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -5083,16 +5032,16 @@
         <v>2</v>
       </c>
       <c r="B116" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C116" s="2">
         <v>115</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="F116">
-        <v>18.060000000000059</v>
+        <v>2142.1</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -5100,16 +5049,16 @@
         <v>2</v>
       </c>
       <c r="B117" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C117" s="2">
         <v>116</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="F117">
-        <v>2.5999999999999996</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -5117,16 +5066,16 @@
         <v>2</v>
       </c>
       <c r="B118" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C118" s="2">
         <v>117</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="F118">
-        <v>17.512999999999998</v>
+        <v>13.065000000000001</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -5134,16 +5083,16 @@
         <v>2</v>
       </c>
       <c r="B119" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C119" s="2">
         <v>118</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="F119">
-        <v>41.523200000000003</v>
+        <v>1.9132000000000033</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -5151,16 +5100,16 @@
         <v>2</v>
       </c>
       <c r="B120" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C120" s="2">
         <v>119</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="F120">
-        <v>16.992800000000006</v>
+        <v>2.7127999999999997</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -5168,13 +5117,13 @@
         <v>2</v>
       </c>
       <c r="B121" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C121" s="2">
         <v>120</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>126</v>
+        <v>98</v>
       </c>
       <c r="F121">
         <v>31.5</v>
@@ -5185,16 +5134,16 @@
         <v>2</v>
       </c>
       <c r="B122" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C122" s="2">
         <v>121</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F122">
-        <v>9.9990000000000023</v>
+        <v>8.958000000000002</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -5202,16 +5151,16 @@
         <v>2</v>
       </c>
       <c r="B123" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C123" s="2">
         <v>122</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="F123">
-        <v>20.891999999999996</v>
+        <v>14.737</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -5219,13 +5168,13 @@
         <v>2</v>
       </c>
       <c r="B124" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C124" s="2">
         <v>123</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>129</v>
+        <v>99</v>
       </c>
       <c r="F124">
         <v>0</v>
@@ -5236,16 +5185,16 @@
         <v>2</v>
       </c>
       <c r="B125" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C125" s="2">
         <v>124</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F125">
-        <v>563.25000000000455</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -5253,16 +5202,16 @@
         <v>2</v>
       </c>
       <c r="B126" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C126" s="2">
         <v>125</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F126">
-        <v>197.68</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -5270,13 +5219,13 @@
         <v>2</v>
       </c>
       <c r="B127" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C127" s="2">
         <v>126</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="F127">
         <v>0</v>
@@ -5287,16 +5236,16 @@
         <v>2</v>
       </c>
       <c r="B128" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C128" s="2">
         <v>127</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="F128">
-        <v>54753</v>
+        <v>91272</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -5304,13 +5253,13 @@
         <v>2</v>
       </c>
       <c r="B129" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C129" s="2">
         <v>128</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
       <c r="F129">
         <v>0</v>
@@ -5321,16 +5270,16 @@
         <v>2</v>
       </c>
       <c r="B130" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C130" s="2">
         <v>129</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>135</v>
+        <v>101</v>
       </c>
       <c r="F130">
-        <v>-563</v>
+        <v>400</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -5338,16 +5287,16 @@
         <v>2</v>
       </c>
       <c r="B131" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C131" s="2">
         <v>130</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="F131">
-        <v>0</v>
+        <v>10755</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -5355,13 +5304,13 @@
         <v>2</v>
       </c>
       <c r="B132" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C132" s="2">
         <v>131</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="F132">
         <v>0</v>
@@ -5372,13 +5321,13 @@
         <v>2</v>
       </c>
       <c r="B133" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C133" s="2">
         <v>132</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F133">
         <v>0</v>
@@ -5389,13 +5338,13 @@
         <v>2</v>
       </c>
       <c r="B134" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C134" s="2">
         <v>133</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F134">
         <v>0</v>
@@ -5406,16 +5355,16 @@
         <v>2</v>
       </c>
       <c r="B135" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C135" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>140</v>
+        <v>102</v>
       </c>
       <c r="F135">
-        <v>2096.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -5423,13 +5372,13 @@
         <v>2</v>
       </c>
       <c r="B136" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C136" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>141</v>
+        <v>103</v>
       </c>
       <c r="F136">
         <v>0</v>
@@ -5440,16 +5389,16 @@
         <v>2</v>
       </c>
       <c r="B137" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C137" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>142</v>
+        <v>104</v>
       </c>
       <c r="F137">
-        <v>15.472999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138" spans="1:6">
@@ -5457,13 +5406,13 @@
         <v>2</v>
       </c>
       <c r="B138" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C138" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>143</v>
+        <v>105</v>
       </c>
       <c r="F138">
         <v>0</v>
@@ -5474,306 +5423,65 @@
         <v>2</v>
       </c>
       <c r="B139" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="C139" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F139">
-        <v>-5.6843418860808015E-14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:6">
-      <c r="A140" s="1">
-        <v>2</v>
-      </c>
-      <c r="B140" t="s">
-        <v>162</v>
-      </c>
-      <c r="C140" s="2">
-        <v>139</v>
-      </c>
-      <c r="D140" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="F140">
-        <v>-4333</v>
-      </c>
+      <c r="A140" s="1"/>
     </row>
     <row r="141" spans="1:6">
-      <c r="A141" s="1">
-        <v>2</v>
-      </c>
-      <c r="B141" t="s">
-        <v>162</v>
-      </c>
-      <c r="C141" s="2">
-        <v>140</v>
-      </c>
-      <c r="D141" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="F141">
-        <v>-2.8421709430404007E-14</v>
-      </c>
+      <c r="A141" s="1"/>
     </row>
     <row r="142" spans="1:6">
-      <c r="A142" s="1">
-        <v>2</v>
-      </c>
-      <c r="B142" t="s">
-        <v>162</v>
-      </c>
-      <c r="C142" s="2">
-        <v>141</v>
-      </c>
-      <c r="D142" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F142">
-        <v>0</v>
-      </c>
+      <c r="A142" s="1"/>
     </row>
     <row r="143" spans="1:6">
-      <c r="A143" s="1">
-        <v>2</v>
-      </c>
-      <c r="B143" t="s">
-        <v>162</v>
-      </c>
-      <c r="C143" s="2">
-        <v>142</v>
-      </c>
-      <c r="D143" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="F143">
-        <v>0</v>
-      </c>
+      <c r="A143" s="1"/>
     </row>
     <row r="144" spans="1:6">
-      <c r="A144" s="1">
-        <v>2</v>
-      </c>
-      <c r="B144" t="s">
-        <v>162</v>
-      </c>
-      <c r="C144" s="2">
-        <v>143</v>
-      </c>
-      <c r="D144" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F144">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6">
-      <c r="A145" s="1">
-        <v>2</v>
-      </c>
-      <c r="B145" t="s">
-        <v>162</v>
-      </c>
-      <c r="C145" s="2">
-        <v>144</v>
-      </c>
-      <c r="D145" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="F145">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6">
-      <c r="A146" s="1">
-        <v>2</v>
-      </c>
-      <c r="B146" t="s">
-        <v>162</v>
-      </c>
-      <c r="C146" s="2">
-        <v>145</v>
-      </c>
-      <c r="D146" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="F146">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" spans="1:6">
-      <c r="A147" s="1">
-        <v>2</v>
-      </c>
-      <c r="B147" t="s">
-        <v>162</v>
-      </c>
-      <c r="C147" s="2">
-        <v>146</v>
-      </c>
-      <c r="D147" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F147">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" spans="1:6">
-      <c r="A148" s="1">
-        <v>2</v>
-      </c>
-      <c r="B148" t="s">
-        <v>162</v>
-      </c>
-      <c r="C148" s="2">
-        <v>147</v>
-      </c>
-      <c r="D148" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="F148">
-        <v>37.459999999999923</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6">
-      <c r="A149" s="1">
-        <v>2</v>
-      </c>
-      <c r="B149" t="s">
-        <v>162</v>
-      </c>
-      <c r="C149" s="2">
-        <v>148</v>
-      </c>
-      <c r="D149" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F149">
-        <v>37.679999999999993</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6">
-      <c r="A150" s="1">
-        <v>2</v>
-      </c>
-      <c r="B150" t="s">
-        <v>162</v>
-      </c>
-      <c r="C150" s="2">
-        <v>149</v>
-      </c>
-      <c r="D150" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="F150">
-        <v>-235.48000000000002</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6">
-      <c r="A151" s="1">
-        <v>2</v>
-      </c>
-      <c r="B151" t="s">
-        <v>162</v>
-      </c>
-      <c r="C151" s="2">
-        <v>150</v>
-      </c>
-      <c r="D151" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="F151">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6">
-      <c r="A152" s="1">
-        <v>2</v>
-      </c>
-      <c r="B152" t="s">
-        <v>162</v>
-      </c>
-      <c r="C152" s="2">
-        <v>151</v>
-      </c>
-      <c r="D152" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="F152">
-        <v>235.48</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6">
-      <c r="A153" s="1">
-        <v>2</v>
-      </c>
-      <c r="B153" t="s">
-        <v>162</v>
-      </c>
-      <c r="C153" s="2">
-        <v>152</v>
-      </c>
-      <c r="D153" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="F153">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6">
-      <c r="A154" s="1">
-        <v>2</v>
-      </c>
-      <c r="B154" t="s">
-        <v>162</v>
-      </c>
-      <c r="C154" s="2">
-        <v>153</v>
-      </c>
-      <c r="D154" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="F154">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" spans="1:6">
-      <c r="A155" s="1">
-        <v>2</v>
-      </c>
-      <c r="B155" t="s">
-        <v>162</v>
-      </c>
-      <c r="C155" s="2">
-        <v>154</v>
-      </c>
-      <c r="D155" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="F155">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6">
-      <c r="A156" s="1">
-        <v>2</v>
-      </c>
-      <c r="B156" t="s">
-        <v>162</v>
-      </c>
-      <c r="C156" s="2">
-        <v>155</v>
-      </c>
-      <c r="D156" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="F156">
-        <v>0</v>
-      </c>
+      <c r="A144" s="1"/>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" s="1"/>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" s="1"/>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147" s="1"/>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148" s="1"/>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" s="1"/>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" s="1"/>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" s="1"/>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" s="1"/>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" s="1"/>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" s="1"/>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>